<commit_message>
Sca Resolver and single quote test cases added
</commit_message>
<xml_diff>
--- a/src/main/resources/ScanTestData.xlsx
+++ b/src/main/resources/ScanTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation Setup\AST Automation\Automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD84E8E-E8EF-4081-9335-854C4AFB1B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1A5044-1B29-49AE-99C6-9B9E5D6AF945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="93">
   <si>
     <t>ScenarioDescription</t>
   </si>
@@ -304,6 +304,15 @@
   </si>
   <si>
     <t>KICS scan with empty Platform</t>
+  </si>
+  <si>
+    <t>SCA scan with valid Sca Resolver Path with Zip Source</t>
+  </si>
+  <si>
+    <t>`--sca-resolver src/main/resources/ScaResolver-win64/ScaResolver.exe</t>
+  </si>
+  <si>
+    <t>Scanning Zip files is not supported by ScaResolver.Please use non-zip source</t>
   </si>
 </sst>
 </file>
@@ -676,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.90625" customWidth="1"/>
@@ -1464,6 +1473,32 @@
       </c>
       <c r="H33" t="s">
         <v>74</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D34" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34" t="s">
+        <v>7</v>
+      </c>
+      <c r="F34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>